<commit_message>
updates the formats of all the downloadables
</commit_message>
<xml_diff>
--- a/TIME TABLE SAMPLE DATA/query(2).xlsx
+++ b/TIME TABLE SAMPLE DATA/query(2).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rajas\OneDrive\Desktop\Timetable\TIME TABLE SAMPLE DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B684C1B-9745-42BF-80B6-3E33EB1D91F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF468F1C-A187-4D04-BBB3-7C84C0D602F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -396,7 +396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.77734375" customWidth="1"/>
@@ -427,108 +427,108 @@
         <v>10</v>
       </c>
       <c r="C2" s="3">
-        <v>0.58333333333333337</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D2" s="3">
-        <v>0.66666666666666663</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>46108</v>
+        <v>46109</v>
       </c>
       <c r="B3">
         <v>10</v>
       </c>
       <c r="C3" s="3">
-        <v>0.625</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D3" s="3">
-        <v>0.64583333333333337</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>46109</v>
+        <v>46111</v>
       </c>
       <c r="B4">
         <v>10</v>
       </c>
       <c r="C4" s="3">
-        <v>0.4861111111111111</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D4" s="3">
-        <v>0.59027777777777779</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
-        <v>46111</v>
+        <v>46112</v>
       </c>
       <c r="B5">
         <v>10</v>
       </c>
       <c r="C5" s="3">
-        <v>0.50694444444444442</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D5" s="3">
-        <v>0.58333333333333337</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="B6">
         <v>10</v>
       </c>
       <c r="C6" s="3">
-        <v>0.45833333333333331</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D6" s="3">
-        <v>0.52777777777777779</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
-        <v>46113</v>
+        <v>46114</v>
       </c>
       <c r="B7">
         <v>10</v>
       </c>
       <c r="C7" s="3">
-        <v>0.4236111111111111</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D7" s="3">
-        <v>0.61805555555555558</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>46114</v>
+        <v>46115</v>
       </c>
       <c r="B8">
         <v>10</v>
       </c>
       <c r="C8" s="3">
-        <v>0.50694444444444442</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D8" s="3">
-        <v>0.63194444444444442</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="2">
-        <v>46115</v>
+        <v>46116</v>
       </c>
       <c r="B9">
         <v>10</v>
       </c>
       <c r="C9" s="3">
-        <v>0.61111111111111116</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="D9" s="3">
-        <v>0.62708333333333333</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -536,13 +536,125 @@
         <v>46116</v>
       </c>
       <c r="B10">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C10" s="3">
-        <v>0.59027777777777779</v>
+        <v>0.41666666666666669</v>
       </c>
       <c r="D10" s="3">
-        <v>0.66666666666666663</v>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>46107</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B12">
+        <v>10</v>
+      </c>
+      <c r="C12" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>46111</v>
+      </c>
+      <c r="B13">
+        <v>10</v>
+      </c>
+      <c r="C13" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>46112</v>
+      </c>
+      <c r="B14">
+        <v>10</v>
+      </c>
+      <c r="C14" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>46113</v>
+      </c>
+      <c r="B15">
+        <v>10</v>
+      </c>
+      <c r="C15" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>46114</v>
+      </c>
+      <c r="B16">
+        <v>10</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>46115</v>
+      </c>
+      <c r="B17">
+        <v>10</v>
+      </c>
+      <c r="C17" s="3">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>46115</v>
+      </c>
+      <c r="B18">
+        <v>10</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.375</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.41666666666666669</v>
       </c>
     </row>
   </sheetData>

</xml_diff>